<commit_message>
Growth report: refresh 15O weekly series through wk202633
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Growth Report/Catalyst_Growth_Report.xlsx
+++ b/Growth Report/Catalyst_Growth_Report.xlsx
@@ -305,12 +305,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Walmart 15O Weekly'!$A$5:$A$29</f>
+              <f>'Walmart 15O Weekly'!$A$5:$A$37</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Walmart 15O Weekly'!$C$5:$C$29</f>
+              <f>'Walmart 15O Weekly'!$C$5:$C$37</f>
             </numRef>
           </val>
         </ser>
@@ -340,12 +340,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Walmart 15O Weekly'!$A$5:$A$29</f>
+              <f>'Walmart 15O Weekly'!$A$5:$A$37</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Walmart 15O Weekly'!$E$5:$E$29</f>
+              <f>'Walmart 15O Weekly'!$E$5:$E$37</f>
             </numRef>
           </val>
         </ser>
@@ -433,12 +433,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Walmart 15O Weekly'!$A$5:$A$29</f>
+              <f>'Walmart 15O Weekly'!$A$5:$A$37</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Walmart 15O Weekly'!$D$5:$D$29</f>
+              <f>'Walmart 15O Weekly'!$D$5:$D$37</f>
             </numRef>
           </val>
         </ser>
@@ -468,12 +468,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Walmart 15O Weekly'!$A$5:$A$29</f>
+              <f>'Walmart 15O Weekly'!$A$5:$A$37</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Walmart 15O Weekly'!$F$5:$F$29</f>
+              <f>'Walmart 15O Weekly'!$F$5:$F$37</f>
             </numRef>
           </val>
         </ser>
@@ -971,7 +971,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:F39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1042,10 +1042,10 @@
         <v>0.238</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>1694.5</v>
+        <v>1185.6</v>
       </c>
       <c r="F5" s="8" t="n">
-        <v>0.4892</v>
+        <v>0.3518</v>
       </c>
     </row>
     <row r="6">
@@ -1062,10 +1062,10 @@
         <v>0.3903</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>1896.3</v>
+        <v>1441.5</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>0.545</v>
+        <v>0.4221</v>
       </c>
     </row>
     <row r="7">
@@ -1082,10 +1082,10 @@
         <v>0.4613</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>2098.2</v>
+        <v>1697.4</v>
       </c>
       <c r="F7" s="8" t="n">
-        <v>0.6007</v>
+        <v>0.4924</v>
       </c>
     </row>
     <row r="8">
@@ -1102,10 +1102,10 @@
         <v>0.6749000000000001</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>2300</v>
+        <v>1953.3</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>0.6564</v>
+        <v>0.5627</v>
       </c>
     </row>
     <row r="9">
@@ -1122,10 +1122,10 @@
         <v>0.882</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>2501.9</v>
+        <v>2209.2</v>
       </c>
       <c r="F9" s="8" t="n">
-        <v>0.7122000000000001</v>
+        <v>0.633</v>
       </c>
     </row>
     <row r="10">
@@ -1142,10 +1142,10 @@
         <v>0.9372</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>2703.8</v>
+        <v>2465.1</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>0.7679</v>
+        <v>0.7033</v>
       </c>
     </row>
     <row r="11">
@@ -1162,10 +1162,10 @@
         <v>0.883</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>2905.6</v>
+        <v>2721</v>
       </c>
       <c r="F11" s="8" t="n">
-        <v>0.8237</v>
+        <v>0.7736</v>
       </c>
     </row>
     <row r="12">
@@ -1182,10 +1182,10 @@
         <v>0.926</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>3107.5</v>
+        <v>2976.8</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>0.8794</v>
+        <v>0.8439</v>
       </c>
     </row>
     <row r="13">
@@ -1202,10 +1202,10 @@
         <v>0.9887</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>3309.3</v>
+        <v>3232.7</v>
       </c>
       <c r="F13" s="8" t="n">
-        <v>0.9351</v>
+        <v>0.9142</v>
       </c>
     </row>
     <row r="14">
@@ -1222,10 +1222,10 @@
         <v>1.0838</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>3511.2</v>
+        <v>3488.6</v>
       </c>
       <c r="F14" s="8" t="n">
-        <v>0.9909</v>
+        <v>0.9845</v>
       </c>
     </row>
     <row r="15">
@@ -1242,10 +1242,10 @@
         <v>1.1782</v>
       </c>
       <c r="E15" s="5" t="n">
-        <v>3713</v>
+        <v>3744.5</v>
       </c>
       <c r="F15" s="8" t="n">
-        <v>1.0466</v>
+        <v>1.0548</v>
       </c>
     </row>
     <row r="16">
@@ -1262,10 +1262,10 @@
         <v>1.2391</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>3914.9</v>
+        <v>4000.4</v>
       </c>
       <c r="F16" s="8" t="n">
-        <v>1.1023</v>
+        <v>1.1251</v>
       </c>
     </row>
     <row r="17">
@@ -1282,10 +1282,10 @@
         <v>1.1713</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>4116.8</v>
+        <v>4256.3</v>
       </c>
       <c r="F17" s="8" t="n">
-        <v>1.1581</v>
+        <v>1.1954</v>
       </c>
     </row>
     <row r="18">
@@ -1302,10 +1302,10 @@
         <v>1.1996</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>4318.6</v>
+        <v>4512.2</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>1.2138</v>
+        <v>1.2657</v>
       </c>
     </row>
     <row r="19">
@@ -1322,10 +1322,10 @@
         <v>1.2939</v>
       </c>
       <c r="E19" s="5" t="n">
-        <v>4520.5</v>
+        <v>4768</v>
       </c>
       <c r="F19" s="8" t="n">
-        <v>1.2696</v>
+        <v>1.336</v>
       </c>
     </row>
     <row r="20">
@@ -1342,10 +1342,10 @@
         <v>1.373</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>4722.3</v>
+        <v>5023.9</v>
       </c>
       <c r="F20" s="8" t="n">
-        <v>1.3253</v>
+        <v>1.4063</v>
       </c>
     </row>
     <row r="21">
@@ -1362,10 +1362,10 @@
         <v>1.3795</v>
       </c>
       <c r="E21" s="5" t="n">
-        <v>4924.2</v>
+        <v>5279.8</v>
       </c>
       <c r="F21" s="8" t="n">
-        <v>1.381</v>
+        <v>1.4766</v>
       </c>
     </row>
     <row r="22">
@@ -1382,10 +1382,10 @@
         <v>1.443</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>5126.1</v>
+        <v>5535.7</v>
       </c>
       <c r="F22" s="8" t="n">
-        <v>1.4368</v>
+        <v>1.5469</v>
       </c>
     </row>
     <row r="23">
@@ -1402,10 +1402,10 @@
         <v>1.4149</v>
       </c>
       <c r="E23" s="5" t="n">
-        <v>5327.9</v>
+        <v>5791.6</v>
       </c>
       <c r="F23" s="8" t="n">
-        <v>1.4925</v>
+        <v>1.6172</v>
       </c>
     </row>
     <row r="24">
@@ -1422,10 +1422,10 @@
         <v>1.4008</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>5529.8</v>
+        <v>6047.5</v>
       </c>
       <c r="F24" s="8" t="n">
-        <v>1.5483</v>
+        <v>1.6875</v>
       </c>
     </row>
     <row r="25">
@@ -1442,10 +1442,10 @@
         <v>1.3632</v>
       </c>
       <c r="E25" s="5" t="n">
-        <v>5731.6</v>
+        <v>6303.4</v>
       </c>
       <c r="F25" s="8" t="n">
-        <v>1.604</v>
+        <v>1.7578</v>
       </c>
     </row>
     <row r="26">
@@ -1462,10 +1462,10 @@
         <v>1.6101</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>5933.5</v>
+        <v>6559.3</v>
       </c>
       <c r="F26" s="8" t="n">
-        <v>1.6597</v>
+        <v>1.8281</v>
       </c>
     </row>
     <row r="27">
@@ -1482,10 +1482,10 @@
         <v>1.4195</v>
       </c>
       <c r="E27" s="5" t="n">
-        <v>6135.3</v>
+        <v>6815.1</v>
       </c>
       <c r="F27" s="8" t="n">
-        <v>1.7155</v>
+        <v>1.8984</v>
       </c>
     </row>
     <row r="28">
@@ -1502,10 +1502,10 @@
         <v>1.8934</v>
       </c>
       <c r="E28" s="5" t="n">
-        <v>6337.2</v>
+        <v>7071</v>
       </c>
       <c r="F28" s="8" t="n">
-        <v>1.7712</v>
+        <v>1.9687</v>
       </c>
     </row>
     <row r="29">
@@ -1522,26 +1522,186 @@
         <v>2.1075</v>
       </c>
       <c r="E29" s="5" t="n">
-        <v>6539.1</v>
+        <v>7326.9</v>
       </c>
       <c r="F29" s="8" t="n">
-        <v>1.827</v>
+        <v>2.039</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="B30" s="7" t="n">
+        <v>46234</v>
+      </c>
+      <c r="C30" s="5" t="n">
+        <v>6601</v>
+      </c>
+      <c r="D30" s="8" t="n">
+        <v>1.8336</v>
+      </c>
+      <c r="E30" s="5" t="n">
+        <v>7582.8</v>
+      </c>
+      <c r="F30" s="8" t="n">
+        <v>2.1093</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="9" t="inlineStr">
+      <c r="A31" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="B31" s="7" t="n">
+        <v>46241</v>
+      </c>
+      <c r="C31" s="5" t="n">
+        <v>6902</v>
+      </c>
+      <c r="D31" s="8" t="n">
+        <v>1.913</v>
+      </c>
+      <c r="E31" s="5" t="n">
+        <v>7838.7</v>
+      </c>
+      <c r="F31" s="8" t="n">
+        <v>2.1796</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="B32" s="7" t="n">
+        <v>46248</v>
+      </c>
+      <c r="C32" s="5" t="n">
+        <v>8494</v>
+      </c>
+      <c r="D32" s="8" t="n">
+        <v>2.3549</v>
+      </c>
+      <c r="E32" s="5" t="n">
+        <v>8094.6</v>
+      </c>
+      <c r="F32" s="8" t="n">
+        <v>2.2499</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="B33" s="7" t="n">
+        <v>46255</v>
+      </c>
+      <c r="C33" s="5" t="n">
+        <v>9268</v>
+      </c>
+      <c r="D33" s="8" t="n">
+        <v>2.5694</v>
+      </c>
+      <c r="E33" s="5" t="n">
+        <v>8350.5</v>
+      </c>
+      <c r="F33" s="8" t="n">
+        <v>2.3202</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="B34" s="7" t="n">
+        <v>46262</v>
+      </c>
+      <c r="C34" s="5" t="n">
+        <v>9613</v>
+      </c>
+      <c r="D34" s="8" t="n">
+        <v>2.6693</v>
+      </c>
+      <c r="E34" s="5" t="n">
+        <v>8606.299999999999</v>
+      </c>
+      <c r="F34" s="8" t="n">
+        <v>2.3905</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="B35" s="7" t="n">
+        <v>46269</v>
+      </c>
+      <c r="C35" s="5" t="n">
+        <v>10112</v>
+      </c>
+      <c r="D35" s="8" t="n">
+        <v>2.8019</v>
+      </c>
+      <c r="E35" s="5" t="n">
+        <v>8862.200000000001</v>
+      </c>
+      <c r="F35" s="8" t="n">
+        <v>2.4608</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="B36" s="7" t="n">
+        <v>46276</v>
+      </c>
+      <c r="C36" s="5" t="n">
+        <v>9943</v>
+      </c>
+      <c r="D36" s="8" t="n">
+        <v>2.7551</v>
+      </c>
+      <c r="E36" s="5" t="n">
+        <v>9118.1</v>
+      </c>
+      <c r="F36" s="8" t="n">
+        <v>2.531</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="n">
+        <v>33</v>
+      </c>
+      <c r="B37" s="7" t="n">
+        <v>46283</v>
+      </c>
+      <c r="C37" s="5" t="n">
+        <v>10382</v>
+      </c>
+      <c r="D37" s="8" t="n">
+        <v>2.8783</v>
+      </c>
+      <c r="E37" s="5" t="n">
+        <v>9374</v>
+      </c>
+      <c r="F37" s="8" t="n">
+        <v>2.6013</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="9" t="inlineStr">
         <is>
           <t>Linear weekly growth:</t>
         </is>
       </c>
-      <c r="C31" s="10" t="inlineStr">
+      <c r="C39" s="10" t="inlineStr">
         <is>
-          <t>+202 units/wk</t>
+          <t>+256 units/wk</t>
         </is>
       </c>
-      <c r="D31" s="10" t="inlineStr">
+      <c r="D39" s="10" t="inlineStr">
         <is>
-          <t>+0.056 U/S/W per wk</t>
+          <t>+0.070 U/S/W per wk</t>
         </is>
       </c>
     </row>

</xml_diff>